<commit_message>
Rebuild blacklist import with configured validation
</commit_message>
<xml_diff>
--- a/prototype/sms-blacklist-import-template.xlsx
+++ b/prototype/sms-blacklist-import-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="黑名单导入" sheetId="1" r:id="Rbad473ed60d443b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="Rc32e14c91ec14994"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="黑名单导入" sheetId="1" r:id="Rd2acef0716c54e8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="Rf433f2773d0a4a6f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -319,7 +319,7 @@
         <x:v>非本人手机号</x:v>
       </x:c>
       <x:c r="E2" s="4" t="str">
-        <x:v>催收系统</x:v>
+        <x:v>租后系统</x:v>
       </x:c>
       <x:c r="F2" s="4" t="str">
         <x:v>客户明确拒收</x:v>
@@ -377,7 +377,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbfa6e6eb7d84f39"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R026d3324510b49ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -435,7 +435,7 @@
         <x:v>来源系统</x:v>
       </x:c>
       <x:c r="B6" s="5" t="str">
-        <x:v>必填；催收系统、法诉系统的数据必须填催收类</x:v>
+        <x:v>必填：租后系统、法诉系统、营销平台、客服系统、大平台系统、租赁系统；租后系统、法诉系统的数据必须填催收类</x:v>
       </x:c>
     </x:row>
     <x:row r="7">

</xml_diff>